<commit_message>
fix(test): use 'Voltage In' for missing-column fixture (no plain 'Voltage' in schema)
</commit_message>
<xml_diff>
--- a/src/lib/__fixtures__/missing-column.xlsx
+++ b/src/lib/__fixtures__/missing-column.xlsx
@@ -927,7 +927,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="858" uniqueCount="479">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="857" uniqueCount="478">
   <si>
     <t>Revision History</t>
   </si>
@@ -1280,9 +1280,6 @@
   </si>
   <si>
     <t>Wire Number (COM Out)</t>
-  </si>
-  <si>
-    <t>Voltage In</t>
   </si>
   <si>
     <t>Amperage In</t>
@@ -4486,33 +4483,33 @@
         <v>110</v>
       </c>
       <c r="I2" s="7" t="s">
+        <v>393</v>
+      </c>
+      <c r="J2" s="7" t="s">
         <v>394</v>
       </c>
-      <c r="J2" s="7" t="s">
+      <c r="K2" s="7" t="s">
         <v>395</v>
       </c>
-      <c r="K2" s="7" t="s">
+      <c r="L2" s="7" t="s">
         <v>396</v>
       </c>
-      <c r="L2" s="7" t="s">
+      <c r="M2" s="4" t="s">
+        <v>122</v>
+      </c>
+      <c r="N2" s="7" t="s">
+        <v>123</v>
+      </c>
+      <c r="O2" s="7" t="s">
         <v>397</v>
       </c>
-      <c r="M2" s="4" t="s">
-        <v>123</v>
-      </c>
-      <c r="N2" s="7" t="s">
-        <v>124</v>
-      </c>
-      <c r="O2" s="7" t="s">
-        <v>398</v>
-      </c>
       <c r="P2" s="8" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
     </row>
     <row r="3" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A3" s="9" t="s">
-        <v>399</v>
+        <v>398</v>
       </c>
       <c r="B3" t="s">
         <v>90</v>
@@ -4521,25 +4518,25 @@
         <v>91</v>
       </c>
       <c r="D3" t="s">
-        <v>385</v>
+        <v>384</v>
       </c>
       <c r="E3" t="s">
-        <v>384</v>
+        <v>383</v>
       </c>
       <c r="F3" t="s">
+        <v>399</v>
+      </c>
+      <c r="G3" t="s">
         <v>400</v>
       </c>
-      <c r="G3" t="s">
+      <c r="H3" t="s">
         <v>401</v>
-      </c>
-      <c r="H3" t="s">
-        <v>402</v>
       </c>
       <c r="I3">
         <v>2</v>
       </c>
       <c r="J3" t="s">
-        <v>403</v>
+        <v>402</v>
       </c>
       <c r="L3" s="10"/>
       <c r="M3" s="11"/>
@@ -4549,7 +4546,7 @@
     </row>
     <row r="4" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A4" s="9" t="s">
-        <v>404</v>
+        <v>403</v>
       </c>
       <c r="B4" t="s">
         <v>90</v>
@@ -4558,25 +4555,25 @@
         <v>91</v>
       </c>
       <c r="D4" t="s">
-        <v>385</v>
+        <v>384</v>
       </c>
       <c r="E4" t="s">
-        <v>384</v>
+        <v>383</v>
       </c>
       <c r="F4" t="s">
+        <v>404</v>
+      </c>
+      <c r="G4" t="s">
         <v>405</v>
       </c>
-      <c r="G4" t="s">
-        <v>406</v>
-      </c>
       <c r="H4" t="s">
-        <v>402</v>
+        <v>401</v>
       </c>
       <c r="I4">
         <v>2</v>
       </c>
       <c r="J4" t="s">
-        <v>407</v>
+        <v>406</v>
       </c>
       <c r="L4" s="10"/>
       <c r="M4" s="11"/>
@@ -4586,7 +4583,7 @@
     </row>
     <row r="5" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A5" s="9" t="s">
-        <v>408</v>
+        <v>407</v>
       </c>
       <c r="B5" t="s">
         <v>90</v>
@@ -4595,25 +4592,25 @@
         <v>91</v>
       </c>
       <c r="D5" t="s">
-        <v>390</v>
+        <v>389</v>
       </c>
       <c r="E5" t="s">
-        <v>384</v>
+        <v>383</v>
       </c>
       <c r="F5" t="s">
+        <v>408</v>
+      </c>
+      <c r="G5" t="s">
         <v>409</v>
       </c>
-      <c r="G5" t="s">
+      <c r="H5" t="s">
         <v>410</v>
-      </c>
-      <c r="H5" t="s">
-        <v>411</v>
       </c>
       <c r="I5">
         <v>2</v>
       </c>
       <c r="J5" t="s">
-        <v>412</v>
+        <v>411</v>
       </c>
       <c r="L5" s="10"/>
       <c r="M5" s="11"/>
@@ -4623,7 +4620,7 @@
     </row>
     <row r="6" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A6" s="9" t="s">
-        <v>413</v>
+        <v>412</v>
       </c>
       <c r="B6" t="s">
         <v>90</v>
@@ -4632,25 +4629,25 @@
         <v>91</v>
       </c>
       <c r="D6" t="s">
-        <v>390</v>
+        <v>389</v>
       </c>
       <c r="E6" t="s">
-        <v>384</v>
+        <v>383</v>
       </c>
       <c r="F6" t="s">
+        <v>413</v>
+      </c>
+      <c r="G6" t="s">
         <v>414</v>
       </c>
-      <c r="G6" t="s">
-        <v>415</v>
-      </c>
       <c r="H6" t="s">
-        <v>411</v>
+        <v>410</v>
       </c>
       <c r="I6">
         <v>2</v>
       </c>
       <c r="J6" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
       <c r="L6" s="10"/>
       <c r="M6" s="11"/>
@@ -4697,23 +4694,23 @@
       </c>
       <c r="B1" s="53"/>
       <c r="C1" s="6" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="D1" s="6"/>
       <c r="E1" s="6" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="F1" s="6"/>
       <c r="G1" s="6" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
       <c r="H1" s="6"/>
       <c r="I1" s="6" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="J1" s="6"/>
       <c r="K1" s="6" t="s">
-        <v>367</v>
+        <v>366</v>
       </c>
       <c r="L1" s="6"/>
     </row>
@@ -4725,34 +4722,34 @@
         <v>109</v>
       </c>
       <c r="C2" s="4" t="s">
+        <v>367</v>
+      </c>
+      <c r="D2" s="8" t="s">
         <v>368</v>
       </c>
-      <c r="D2" s="8" t="s">
+      <c r="E2" s="4" t="s">
         <v>369</v>
       </c>
-      <c r="E2" s="4" t="s">
+      <c r="F2" s="8" t="s">
         <v>370</v>
       </c>
-      <c r="F2" s="8" t="s">
+      <c r="G2" s="4" t="s">
         <v>371</v>
       </c>
-      <c r="G2" s="4" t="s">
+      <c r="H2" s="8" t="s">
         <v>372</v>
       </c>
-      <c r="H2" s="8" t="s">
+      <c r="I2" s="4" t="s">
         <v>373</v>
       </c>
-      <c r="I2" s="4" t="s">
+      <c r="J2" s="8" t="s">
         <v>374</v>
       </c>
-      <c r="J2" s="8" t="s">
+      <c r="K2" s="4" t="s">
         <v>375</v>
       </c>
-      <c r="K2" s="4" t="s">
+      <c r="L2" s="8" t="s">
         <v>376</v>
-      </c>
-      <c r="L2" s="8" t="s">
-        <v>377</v>
       </c>
     </row>
     <row r="3" spans="1:12" x14ac:dyDescent="0.25">
@@ -4760,7 +4757,7 @@
         <v>90</v>
       </c>
       <c r="B3" s="10" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="C3" s="11">
         <v>6.4</v>
@@ -4782,7 +4779,7 @@
         <v>90</v>
       </c>
       <c r="B4" s="10" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="C4" s="11">
         <v>27.1</v>
@@ -4845,7 +4842,7 @@
       <c r="E1" s="16"/>
       <c r="F1" s="15"/>
       <c r="G1" s="15" t="s">
-        <v>417</v>
+        <v>416</v>
       </c>
       <c r="H1" s="16"/>
       <c r="I1" s="16"/>
@@ -4865,34 +4862,34 @@
         <v>45</v>
       </c>
       <c r="D2" s="7" t="s">
+        <v>417</v>
+      </c>
+      <c r="E2" s="7" t="s">
+        <v>143</v>
+      </c>
+      <c r="F2" s="1" t="s">
+        <v>260</v>
+      </c>
+      <c r="G2" s="19" t="s">
         <v>418</v>
       </c>
-      <c r="E2" s="7" t="s">
-        <v>144</v>
-      </c>
-      <c r="F2" s="1" t="s">
-        <v>261</v>
-      </c>
-      <c r="G2" s="19" t="s">
+      <c r="H2" s="7" t="s">
         <v>419</v>
       </c>
-      <c r="H2" s="7" t="s">
+      <c r="I2" s="7" t="s">
         <v>420</v>
       </c>
-      <c r="I2" s="7" t="s">
+      <c r="J2" s="7" t="s">
         <v>421</v>
       </c>
-      <c r="J2" s="7" t="s">
+      <c r="K2" s="7" t="s">
         <v>422</v>
       </c>
-      <c r="K2" s="7" t="s">
+      <c r="L2" s="7" t="s">
         <v>423</v>
       </c>
-      <c r="L2" s="7" t="s">
+      <c r="M2" s="1" t="s">
         <v>424</v>
-      </c>
-      <c r="M2" s="1" t="s">
-        <v>425</v>
       </c>
     </row>
     <row r="3" spans="1:13" x14ac:dyDescent="0.25">
@@ -4900,38 +4897,38 @@
         <v>79</v>
       </c>
       <c r="B3" s="7" t="s">
+        <v>425</v>
+      </c>
+      <c r="C3" s="7" t="s">
         <v>426</v>
       </c>
-      <c r="C3" s="7" t="s">
+      <c r="D3" s="7" t="s">
+        <v>188</v>
+      </c>
+      <c r="E3" s="7" t="s">
+        <v>157</v>
+      </c>
+      <c r="F3" s="1" t="s">
+        <v>158</v>
+      </c>
+      <c r="G3" s="7" t="s">
         <v>427</v>
       </c>
-      <c r="D3" s="7" t="s">
-        <v>189</v>
-      </c>
-      <c r="E3" s="7" t="s">
-        <v>158</v>
-      </c>
-      <c r="F3" s="1" t="s">
-        <v>159</v>
-      </c>
-      <c r="G3" s="7" t="s">
+      <c r="H3" s="7" t="s">
         <v>428</v>
       </c>
-      <c r="H3" s="7" t="s">
+      <c r="I3" s="7" t="s">
         <v>429</v>
-      </c>
-      <c r="I3" s="7" t="s">
-        <v>430</v>
       </c>
       <c r="J3" s="7"/>
       <c r="K3" s="7" t="s">
+        <v>430</v>
+      </c>
+      <c r="L3" s="7" t="s">
         <v>431</v>
       </c>
-      <c r="L3" s="7" t="s">
+      <c r="M3" s="7" t="s">
         <v>432</v>
-      </c>
-      <c r="M3" s="7" t="s">
-        <v>433</v>
       </c>
     </row>
     <row r="4" spans="1:13" x14ac:dyDescent="0.25">
@@ -4939,38 +4936,38 @@
         <v>79</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>426</v>
+        <v>425</v>
       </c>
       <c r="C4" s="7" t="s">
+        <v>433</v>
+      </c>
+      <c r="D4" s="7" t="s">
+        <v>188</v>
+      </c>
+      <c r="E4" s="7" t="s">
+        <v>157</v>
+      </c>
+      <c r="F4" s="1" t="s">
+        <v>158</v>
+      </c>
+      <c r="G4" s="7" t="s">
         <v>434</v>
       </c>
-      <c r="D4" s="7" t="s">
-        <v>189</v>
-      </c>
-      <c r="E4" s="7" t="s">
-        <v>158</v>
-      </c>
-      <c r="F4" s="1" t="s">
-        <v>159</v>
-      </c>
-      <c r="G4" s="7" t="s">
+      <c r="H4" s="7" t="s">
         <v>435</v>
       </c>
-      <c r="H4" s="7" t="s">
+      <c r="I4" s="7" t="s">
         <v>436</v>
-      </c>
-      <c r="I4" s="7" t="s">
-        <v>437</v>
       </c>
       <c r="J4" s="7"/>
       <c r="K4" s="7" t="s">
+        <v>437</v>
+      </c>
+      <c r="L4" s="7" t="s">
         <v>438</v>
       </c>
-      <c r="L4" s="7" t="s">
+      <c r="M4" s="7" t="s">
         <v>439</v>
-      </c>
-      <c r="M4" s="7" t="s">
-        <v>440</v>
       </c>
     </row>
   </sheetData>
@@ -5021,14 +5018,14 @@
       <c r="G1" s="7"/>
       <c r="H1" s="6"/>
       <c r="I1" s="16" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="J1" s="17"/>
       <c r="K1" s="17"/>
       <c r="L1" s="17"/>
       <c r="M1" s="18"/>
       <c r="N1" s="6" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="O1" s="7"/>
       <c r="P1" s="7"/>
@@ -5046,10 +5043,10 @@
         <v>42</v>
       </c>
       <c r="B2" s="7" t="s">
+        <v>320</v>
+      </c>
+      <c r="C2" s="7" t="s">
         <v>321</v>
-      </c>
-      <c r="C2" s="7" t="s">
-        <v>322</v>
       </c>
       <c r="D2" s="7" t="s">
         <v>43</v>
@@ -5058,28 +5055,28 @@
         <v>44</v>
       </c>
       <c r="F2" s="7" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="G2" s="7" t="s">
         <v>110</v>
       </c>
       <c r="H2" s="8" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
       <c r="I2" s="19" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="J2" s="7" t="s">
+        <v>147</v>
+      </c>
+      <c r="K2" s="7" t="s">
+        <v>120</v>
+      </c>
+      <c r="L2" s="7" t="s">
+        <v>121</v>
+      </c>
+      <c r="M2" s="1" t="s">
         <v>148</v>
-      </c>
-      <c r="K2" s="7" t="s">
-        <v>121</v>
-      </c>
-      <c r="L2" s="7" t="s">
-        <v>122</v>
-      </c>
-      <c r="M2" s="1" t="s">
-        <v>149</v>
       </c>
       <c r="N2" s="4" t="s">
         <v>58</v>
@@ -5100,18 +5097,18 @@
         <v>63</v>
       </c>
       <c r="T2" s="4" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="U2" s="7" t="s">
+        <v>324</v>
+      </c>
+      <c r="V2" s="8" t="s">
         <v>325</v>
-      </c>
-      <c r="V2" s="8" t="s">
-        <v>326</v>
       </c>
     </row>
     <row r="3" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A3" s="9" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
       <c r="B3" s="1" t="b">
         <v>1</v>
@@ -5126,37 +5123,37 @@
         <v>80</v>
       </c>
       <c r="F3" t="s">
+        <v>327</v>
+      </c>
+      <c r="G3" t="s">
         <v>328</v>
-      </c>
-      <c r="G3" t="s">
-        <v>329</v>
       </c>
       <c r="H3" s="10">
         <v>10</v>
       </c>
       <c r="I3" s="11" t="s">
+        <v>329</v>
+      </c>
+      <c r="J3" t="s">
+        <v>137</v>
+      </c>
+      <c r="K3" t="s">
         <v>330</v>
       </c>
-      <c r="J3" t="s">
-        <v>138</v>
-      </c>
-      <c r="K3" t="s">
+      <c r="L3" t="s">
         <v>331</v>
       </c>
-      <c r="L3" t="s">
+      <c r="M3" s="10" t="s">
         <v>332</v>
       </c>
-      <c r="M3" s="10" t="s">
+      <c r="N3" s="11" t="s">
         <v>333</v>
       </c>
-      <c r="N3" s="11" t="s">
+      <c r="O3" t="s">
         <v>334</v>
       </c>
-      <c r="O3" t="s">
+      <c r="P3" t="s">
         <v>335</v>
-      </c>
-      <c r="P3" t="s">
-        <v>336</v>
       </c>
       <c r="S3" s="10"/>
       <c r="T3" s="11"/>
@@ -5165,7 +5162,7 @@
     </row>
     <row r="4" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A4" s="9" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="B4" s="1" t="b">
         <v>1</v>
@@ -5180,25 +5177,25 @@
         <v>102</v>
       </c>
       <c r="F4" t="s">
+        <v>337</v>
+      </c>
+      <c r="G4" t="s">
         <v>338</v>
-      </c>
-      <c r="G4" t="s">
-        <v>339</v>
       </c>
       <c r="H4" s="10">
         <v>8</v>
       </c>
       <c r="I4" s="11" t="s">
+        <v>329</v>
+      </c>
+      <c r="J4" t="s">
+        <v>137</v>
+      </c>
+      <c r="K4" t="s">
         <v>330</v>
       </c>
-      <c r="J4" t="s">
-        <v>138</v>
-      </c>
-      <c r="K4" t="s">
+      <c r="L4" t="s">
         <v>331</v>
-      </c>
-      <c r="L4" t="s">
-        <v>332</v>
       </c>
       <c r="M4" s="10"/>
       <c r="N4" s="11"/>
@@ -5251,7 +5248,7 @@
       <c r="B1" s="16"/>
       <c r="C1" s="53"/>
       <c r="D1" s="6" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
       <c r="E1" s="7"/>
       <c r="F1" s="7"/>
@@ -5281,55 +5278,55 @@
         <v>109</v>
       </c>
       <c r="D2" s="4" t="s">
+        <v>340</v>
+      </c>
+      <c r="E2" s="7" t="s">
         <v>341</v>
       </c>
-      <c r="E2" s="7" t="s">
+      <c r="F2" s="7" t="s">
         <v>342</v>
       </c>
-      <c r="F2" s="7" t="s">
+      <c r="G2" s="7" t="s">
         <v>343</v>
       </c>
-      <c r="G2" s="7" t="s">
+      <c r="H2" s="7" t="s">
         <v>344</v>
       </c>
-      <c r="H2" s="7" t="s">
+      <c r="I2" s="7" t="s">
         <v>345</v>
       </c>
-      <c r="I2" s="7" t="s">
+      <c r="J2" s="8" t="s">
         <v>346</v>
       </c>
-      <c r="J2" s="8" t="s">
+      <c r="K2" s="8" t="s">
         <v>347</v>
       </c>
-      <c r="K2" s="8" t="s">
+      <c r="L2" s="8" t="s">
         <v>348</v>
       </c>
-      <c r="L2" s="8" t="s">
+      <c r="M2" s="8" t="s">
         <v>349</v>
       </c>
-      <c r="M2" s="8" t="s">
+      <c r="N2" s="8" t="s">
         <v>350</v>
       </c>
-      <c r="N2" s="8" t="s">
+      <c r="O2" s="8" t="s">
         <v>351</v>
       </c>
-      <c r="O2" s="8" t="s">
+      <c r="P2" s="8" t="s">
         <v>352</v>
       </c>
-      <c r="P2" s="8" t="s">
+      <c r="Q2" s="8" t="s">
         <v>353</v>
       </c>
-      <c r="Q2" s="8" t="s">
+      <c r="R2" s="8" t="s">
         <v>354</v>
       </c>
-      <c r="R2" s="8" t="s">
+      <c r="S2" s="8" t="s">
         <v>355</v>
       </c>
-      <c r="S2" s="8" t="s">
+      <c r="T2" s="8" t="s">
         <v>356</v>
-      </c>
-      <c r="T2" s="8" t="s">
-        <v>357</v>
       </c>
     </row>
     <row r="3" spans="1:20" x14ac:dyDescent="0.25">
@@ -5340,7 +5337,7 @@
         <v>91</v>
       </c>
       <c r="C3" s="10" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="D3" s="11">
         <v>460</v>
@@ -5360,13 +5357,13 @@
         <v>100</v>
       </c>
       <c r="K3" t="s">
+        <v>357</v>
+      </c>
+      <c r="L3" t="s">
         <v>358</v>
       </c>
-      <c r="L3" t="s">
+      <c r="M3" t="s">
         <v>359</v>
-      </c>
-      <c r="M3" t="s">
-        <v>360</v>
       </c>
       <c r="N3">
         <v>10</v>
@@ -5385,7 +5382,7 @@
         <v>91</v>
       </c>
       <c r="C4" s="10" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="D4" s="11">
         <v>460</v>
@@ -5405,13 +5402,13 @@
         <v>100</v>
       </c>
       <c r="K4" t="s">
-        <v>358</v>
+        <v>357</v>
       </c>
       <c r="L4" t="s">
+        <v>360</v>
+      </c>
+      <c r="M4" t="s">
         <v>361</v>
-      </c>
-      <c r="M4" t="s">
-        <v>362</v>
       </c>
       <c r="N4">
         <v>10</v>
@@ -5522,12 +5519,12 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="56" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" s="57" t="s">
-        <v>442</v>
+        <v>441</v>
       </c>
       <c r="B2" s="57"/>
       <c r="C2" s="57"/>
@@ -5535,13 +5532,13 @@
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" s="56" t="s">
+        <v>442</v>
+      </c>
+      <c r="B4" s="56" t="s">
         <v>443</v>
       </c>
-      <c r="B4" s="56" t="s">
+      <c r="C4" s="56" t="s">
         <v>444</v>
-      </c>
-      <c r="C4" s="56" t="s">
-        <v>445</v>
       </c>
       <c r="D4" s="56" t="s">
         <v>5</v>
@@ -5549,21 +5546,21 @@
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>446</v>
+        <v>445</v>
       </c>
       <c r="B5" t="s">
         <v>80</v>
       </c>
       <c r="C5" t="s">
+        <v>446</v>
+      </c>
+      <c r="D5" s="57" t="s">
         <v>447</v>
-      </c>
-      <c r="D5" s="57" t="s">
-        <v>448</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>446</v>
+        <v>445</v>
       </c>
       <c r="B6" t="s">
         <v>80</v>
@@ -5572,12 +5569,12 @@
         <v>80</v>
       </c>
       <c r="D6" s="57" t="s">
-        <v>449</v>
+        <v>448</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>446</v>
+        <v>445</v>
       </c>
       <c r="B7" t="s">
         <v>91</v>
@@ -5586,12 +5583,12 @@
         <v>91</v>
       </c>
       <c r="D7" s="57" t="s">
-        <v>450</v>
+        <v>449</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="B8" t="s">
         <v>91</v>
@@ -5600,147 +5597,147 @@
         <v>91</v>
       </c>
       <c r="D8" s="57" t="s">
-        <v>451</v>
+        <v>450</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>452</v>
+        <v>451</v>
       </c>
       <c r="B9" t="s">
         <v>80</v>
       </c>
       <c r="C9" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="D9" s="57" t="s">
-        <v>453</v>
+        <v>452</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>452</v>
+        <v>451</v>
       </c>
       <c r="B10" t="s">
         <v>91</v>
       </c>
       <c r="C10" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="D10" s="57" t="s">
-        <v>454</v>
+        <v>453</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>455</v>
+        <v>454</v>
       </c>
       <c r="B11" t="s">
         <v>80</v>
       </c>
       <c r="C11" t="s">
+        <v>455</v>
+      </c>
+      <c r="D11" s="57" t="s">
         <v>456</v>
-      </c>
-      <c r="D11" s="57" t="s">
-        <v>457</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>455</v>
+        <v>454</v>
       </c>
       <c r="B12" t="s">
         <v>80</v>
       </c>
       <c r="C12" t="s">
+        <v>457</v>
+      </c>
+      <c r="D12" s="57" t="s">
         <v>458</v>
-      </c>
-      <c r="D12" s="57" t="s">
-        <v>459</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>455</v>
+        <v>454</v>
       </c>
       <c r="B13" t="s">
         <v>80</v>
       </c>
       <c r="C13" t="s">
+        <v>459</v>
+      </c>
+      <c r="D13" s="57" t="s">
         <v>460</v>
-      </c>
-      <c r="D13" s="57" t="s">
-        <v>461</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>455</v>
+        <v>454</v>
       </c>
       <c r="B14" t="s">
         <v>80</v>
       </c>
       <c r="C14" t="s">
+        <v>461</v>
+      </c>
+      <c r="D14" s="57" t="s">
         <v>462</v>
-      </c>
-      <c r="D14" s="57" t="s">
-        <v>463</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>464</v>
+        <v>463</v>
       </c>
       <c r="B15" t="s">
         <v>91</v>
       </c>
       <c r="C15" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="D15" s="57" t="s">
-        <v>465</v>
+        <v>464</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>464</v>
+        <v>463</v>
       </c>
       <c r="B16" t="s">
         <v>91</v>
       </c>
       <c r="C16" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="D16" s="57" t="s">
-        <v>466</v>
+        <v>465</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>467</v>
+        <v>466</v>
       </c>
       <c r="B17" t="s">
         <v>91</v>
       </c>
       <c r="C17" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="D17" s="57" t="s">
-        <v>468</v>
+        <v>467</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>467</v>
+        <v>466</v>
       </c>
       <c r="B18" t="s">
         <v>102</v>
       </c>
       <c r="C18" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="D18" s="57" t="s">
-        <v>469</v>
+        <v>468</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.25">
@@ -5751,10 +5748,10 @@
         <v>80</v>
       </c>
       <c r="C19" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="D19" s="57" t="s">
-        <v>470</v>
+        <v>469</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.25">
@@ -5765,38 +5762,38 @@
         <v>91</v>
       </c>
       <c r="C20" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="D20" s="57" t="s">
-        <v>471</v>
+        <v>470</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>472</v>
+        <v>471</v>
       </c>
       <c r="B21" t="s">
         <v>102</v>
       </c>
       <c r="C21" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="D21" s="57" t="s">
-        <v>473</v>
+        <v>472</v>
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>474</v>
+        <v>473</v>
       </c>
       <c r="B22" t="s">
         <v>91</v>
       </c>
       <c r="C22" t="s">
-        <v>447</v>
+        <v>446</v>
       </c>
       <c r="D22" s="57" t="s">
-        <v>475</v>
+        <v>474</v>
       </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.25">
@@ -5807,10 +5804,10 @@
         <v>91</v>
       </c>
       <c r="C23" t="s">
-        <v>385</v>
+        <v>384</v>
       </c>
       <c r="D23" s="57" t="s">
-        <v>476</v>
+        <v>475</v>
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.25">
@@ -5821,10 +5818,10 @@
         <v>91</v>
       </c>
       <c r="C24" t="s">
-        <v>390</v>
+        <v>389</v>
       </c>
       <c r="D24" s="57" t="s">
-        <v>477</v>
+        <v>476</v>
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.25">
@@ -5835,10 +5832,10 @@
         <v>80</v>
       </c>
       <c r="C25" t="s">
-        <v>426</v>
+        <v>425</v>
       </c>
       <c r="D25" s="57" t="s">
-        <v>478</v>
+        <v>477</v>
       </c>
     </row>
   </sheetData>
@@ -5891,19 +5888,19 @@
       <c r="I1" s="16"/>
       <c r="J1" s="15"/>
       <c r="K1" s="16" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="L1" s="17"/>
       <c r="M1" s="17"/>
       <c r="N1" s="17"/>
       <c r="O1" s="18"/>
       <c r="P1" s="16" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="Q1" s="17"/>
       <c r="R1" s="18"/>
       <c r="S1" s="16" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="T1" s="17"/>
       <c r="U1" s="17"/>
@@ -5923,7 +5920,7 @@
         <v>42</v>
       </c>
       <c r="B2" s="20" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="C2" s="20" t="s">
         <v>43</v>
@@ -5932,7 +5929,7 @@
         <v>44</v>
       </c>
       <c r="E2" s="7" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="F2" s="7" t="s">
         <v>45</v>
@@ -5941,28 +5938,28 @@
         <v>110</v>
       </c>
       <c r="H2" s="7" t="s">
+        <v>143</v>
+      </c>
+      <c r="I2" s="7" t="s">
         <v>144</v>
       </c>
-      <c r="I2" s="7" t="s">
+      <c r="J2" s="7" t="s">
         <v>145</v>
       </c>
-      <c r="J2" s="7" t="s">
+      <c r="K2" s="19" t="s">
         <v>146</v>
       </c>
-      <c r="K2" s="19" t="s">
+      <c r="L2" s="7" t="s">
         <v>147</v>
       </c>
-      <c r="L2" s="7" t="s">
+      <c r="M2" s="7" t="s">
+        <v>120</v>
+      </c>
+      <c r="N2" s="7" t="s">
+        <v>121</v>
+      </c>
+      <c r="O2" s="1" t="s">
         <v>148</v>
-      </c>
-      <c r="M2" s="7" t="s">
-        <v>121</v>
-      </c>
-      <c r="N2" s="7" t="s">
-        <v>122</v>
-      </c>
-      <c r="O2" s="1" t="s">
-        <v>149</v>
       </c>
       <c r="P2" s="19" t="s">
         <v>54</v>
@@ -5992,24 +5989,24 @@
         <v>63</v>
       </c>
       <c r="Y2" s="19" t="s">
+        <v>149</v>
+      </c>
+      <c r="Z2" s="7" t="s">
         <v>150</v>
       </c>
-      <c r="Z2" s="7" t="s">
+      <c r="AA2" s="7" t="s">
         <v>151</v>
       </c>
-      <c r="AA2" s="7" t="s">
+      <c r="AB2" s="7" t="s">
         <v>152</v>
       </c>
-      <c r="AB2" s="7" t="s">
-        <v>153</v>
-      </c>
       <c r="AC2" s="1" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
     </row>
     <row r="3" spans="1:29" s="7" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A3" s="9" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="B3" s="20" t="b">
         <v>1</v>
@@ -6021,35 +6018,35 @@
         <v>80</v>
       </c>
       <c r="E3" s="7" t="s">
+        <v>154</v>
+      </c>
+      <c r="F3" s="7" t="s">
         <v>155</v>
       </c>
-      <c r="F3" s="7" t="s">
+      <c r="G3" s="7" t="s">
         <v>156</v>
       </c>
-      <c r="G3" s="7" t="s">
+      <c r="H3" s="7" t="s">
         <v>157</v>
       </c>
-      <c r="H3" s="7" t="s">
+      <c r="I3" s="7" t="s">
         <v>158</v>
-      </c>
-      <c r="I3" s="7" t="s">
-        <v>159</v>
       </c>
       <c r="J3" s="1"/>
       <c r="K3" s="19" t="s">
+        <v>159</v>
+      </c>
+      <c r="L3" s="7" t="s">
+        <v>128</v>
+      </c>
+      <c r="M3" s="7" t="s">
+        <v>129</v>
+      </c>
+      <c r="N3" s="7" t="s">
+        <v>130</v>
+      </c>
+      <c r="O3" s="1" t="s">
         <v>160</v>
-      </c>
-      <c r="L3" s="7" t="s">
-        <v>129</v>
-      </c>
-      <c r="M3" s="7" t="s">
-        <v>130</v>
-      </c>
-      <c r="N3" s="7" t="s">
-        <v>131</v>
-      </c>
-      <c r="O3" s="1" t="s">
-        <v>161</v>
       </c>
       <c r="P3" s="19"/>
       <c r="Q3" s="7"/>
@@ -6068,7 +6065,7 @@
     </row>
     <row r="4" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A4" s="9" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="B4" s="20" t="b">
         <v>0</v>
@@ -6080,37 +6077,37 @@
         <v>91</v>
       </c>
       <c r="E4" s="7" t="s">
+        <v>162</v>
+      </c>
+      <c r="F4" s="7" t="s">
         <v>163</v>
       </c>
-      <c r="F4" s="7" t="s">
+      <c r="G4" s="7" t="s">
         <v>164</v>
       </c>
-      <c r="G4" s="7" t="s">
+      <c r="H4" s="7" t="s">
         <v>165</v>
       </c>
-      <c r="H4" s="7" t="s">
+      <c r="I4" s="7" t="s">
+        <v>158</v>
+      </c>
+      <c r="J4" s="1" t="s">
         <v>166</v>
       </c>
-      <c r="I4" s="7" t="s">
-        <v>159</v>
-      </c>
-      <c r="J4" s="1" t="s">
+      <c r="K4" s="19" t="s">
         <v>167</v>
       </c>
-      <c r="K4" s="19" t="s">
+      <c r="L4" s="7" t="s">
+        <v>137</v>
+      </c>
+      <c r="M4" s="7" t="s">
         <v>168</v>
       </c>
-      <c r="L4" s="7" t="s">
-        <v>138</v>
-      </c>
-      <c r="M4" s="7" t="s">
+      <c r="N4" s="7" t="s">
         <v>169</v>
       </c>
-      <c r="N4" s="7" t="s">
+      <c r="O4" s="1" t="s">
         <v>170</v>
-      </c>
-      <c r="O4" s="1" t="s">
-        <v>171</v>
       </c>
       <c r="P4" s="19"/>
       <c r="Q4" s="7"/>
@@ -6244,40 +6241,38 @@
       <c r="L2" s="8" t="s">
         <v>116</v>
       </c>
-      <c r="M2" s="4" t="s">
+      <c r="M2" s="4"/>
+      <c r="N2" s="7" t="s">
         <v>117</v>
       </c>
-      <c r="N2" s="7" t="s">
+      <c r="O2" s="7" t="s">
         <v>118</v>
       </c>
-      <c r="O2" s="7" t="s">
+      <c r="P2" s="7" t="s">
         <v>119</v>
       </c>
-      <c r="P2" s="7" t="s">
+      <c r="Q2" s="7" t="s">
         <v>120</v>
       </c>
-      <c r="Q2" s="7" t="s">
+      <c r="R2" s="8" t="s">
         <v>121</v>
       </c>
-      <c r="R2" s="8" t="s">
+      <c r="S2" s="4" t="s">
         <v>122</v>
       </c>
-      <c r="S2" s="4" t="s">
+      <c r="T2" s="7" t="s">
         <v>123</v>
       </c>
-      <c r="T2" s="7" t="s">
+      <c r="U2" s="7" t="s">
         <v>124</v>
       </c>
-      <c r="U2" s="7" t="s">
+      <c r="V2" s="8" t="s">
         <v>125</v>
-      </c>
-      <c r="V2" s="8" t="s">
-        <v>126</v>
       </c>
     </row>
     <row r="3" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A3" s="9" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="B3" s="8" t="s">
         <v>79</v>
@@ -6286,27 +6281,27 @@
         <v>80</v>
       </c>
       <c r="D3" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="G3" s="10"/>
       <c r="H3" s="11" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="J3" t="s">
         <v>84</v>
       </c>
       <c r="L3" s="10"/>
       <c r="M3" s="11" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="O3" t="s">
         <v>84</v>
       </c>
       <c r="Q3" t="s">
+        <v>129</v>
+      </c>
+      <c r="R3" s="10" t="s">
         <v>130</v>
-      </c>
-      <c r="R3" s="10" t="s">
-        <v>131</v>
       </c>
       <c r="S3" s="11"/>
       <c r="T3" s="1"/>
@@ -6315,7 +6310,7 @@
     </row>
     <row r="4" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A4" s="9" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="B4" s="8" t="s">
         <v>90</v>
@@ -6324,11 +6319,11 @@
         <v>91</v>
       </c>
       <c r="D4" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="G4" s="10"/>
       <c r="H4" s="11" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="I4">
         <v>10</v>
@@ -6338,7 +6333,7 @@
       </c>
       <c r="L4" s="10"/>
       <c r="M4" s="11" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="N4">
         <v>30</v>
@@ -6354,7 +6349,7 @@
     </row>
     <row r="5" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A5" s="9" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="B5" s="8" t="s">
         <v>90</v>
@@ -6363,14 +6358,14 @@
         <v>91</v>
       </c>
       <c r="E5" t="s">
+        <v>135</v>
+      </c>
+      <c r="F5" t="s">
         <v>136</v>
-      </c>
-      <c r="F5" t="s">
-        <v>137</v>
       </c>
       <c r="G5" s="10"/>
       <c r="H5" s="11" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="I5">
         <v>5</v>
@@ -6380,7 +6375,7 @@
       </c>
       <c r="L5" s="10"/>
       <c r="M5" s="11" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="O5" t="s">
         <v>84</v>
@@ -6452,7 +6447,7 @@
       <c r="H1" s="21"/>
       <c r="I1" s="22"/>
       <c r="J1" s="18" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="K1" s="21"/>
       <c r="L1" s="21"/>
@@ -6461,7 +6456,7 @@
       <c r="O1" s="21"/>
       <c r="P1" s="22"/>
       <c r="Q1" s="18" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="R1" s="21"/>
       <c r="S1" s="21"/>
@@ -6481,7 +6476,7 @@
         <v>107</v>
       </c>
       <c r="B2" s="7" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="C2" s="7" t="s">
         <v>43</v>
@@ -6490,7 +6485,7 @@
         <v>44</v>
       </c>
       <c r="E2" s="7" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="F2" s="7" t="s">
         <v>45</v>
@@ -6499,69 +6494,69 @@
         <v>110</v>
       </c>
       <c r="H2" s="7" t="s">
+        <v>173</v>
+      </c>
+      <c r="I2" s="1" t="s">
         <v>174</v>
-      </c>
-      <c r="I2" s="1" t="s">
-        <v>175</v>
       </c>
       <c r="J2" s="25" t="s">
         <v>111</v>
       </c>
       <c r="K2" s="25" t="s">
+        <v>147</v>
+      </c>
+      <c r="L2" s="25" t="s">
+        <v>175</v>
+      </c>
+      <c r="M2" s="25" t="s">
+        <v>120</v>
+      </c>
+      <c r="N2" s="25" t="s">
+        <v>176</v>
+      </c>
+      <c r="O2" s="25" t="s">
+        <v>121</v>
+      </c>
+      <c r="P2" s="26" t="s">
         <v>148</v>
       </c>
-      <c r="L2" s="25" t="s">
-        <v>176</v>
-      </c>
-      <c r="M2" s="25" t="s">
-        <v>121</v>
-      </c>
-      <c r="N2" s="25" t="s">
+      <c r="Q2" s="25" t="s">
         <v>177</v>
       </c>
-      <c r="O2" s="25" t="s">
-        <v>122</v>
-      </c>
-      <c r="P2" s="26" t="s">
-        <v>149</v>
-      </c>
-      <c r="Q2" s="25" t="s">
+      <c r="R2" s="25" t="s">
         <v>178</v>
       </c>
-      <c r="R2" s="25" t="s">
+      <c r="S2" s="25" t="s">
         <v>179</v>
       </c>
-      <c r="S2" s="25" t="s">
+      <c r="T2" s="25" t="s">
         <v>180</v>
       </c>
-      <c r="T2" s="25" t="s">
+      <c r="U2" s="25" t="s">
         <v>181</v>
       </c>
-      <c r="U2" s="25" t="s">
+      <c r="V2" s="25" t="s">
         <v>182</v>
       </c>
-      <c r="V2" s="25" t="s">
+      <c r="W2" s="26" t="s">
         <v>183</v>
       </c>
-      <c r="W2" s="26" t="s">
+      <c r="X2" s="19" t="s">
         <v>184</v>
       </c>
-      <c r="X2" s="19" t="s">
+      <c r="Y2" s="7" t="s">
+        <v>123</v>
+      </c>
+      <c r="Z2" s="7" t="s">
         <v>185</v>
       </c>
-      <c r="Y2" s="7" t="s">
-        <v>124</v>
-      </c>
-      <c r="Z2" s="7" t="s">
-        <v>186</v>
-      </c>
       <c r="AA2" s="1" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
     </row>
     <row r="3" spans="1:27" s="7" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A3" s="9" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="B3" s="7" t="b">
         <v>1</v>
@@ -6573,13 +6568,13 @@
         <v>80</v>
       </c>
       <c r="E3" s="7" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="F3" s="7" t="s">
+        <v>187</v>
+      </c>
+      <c r="G3" s="7" t="s">
         <v>188</v>
-      </c>
-      <c r="G3" s="7" t="s">
-        <v>189</v>
       </c>
       <c r="H3" s="7">
         <v>32.013</v>
@@ -6608,7 +6603,7 @@
     </row>
     <row r="4" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A4" s="9" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="B4" s="7" t="b">
         <v>1</v>
@@ -6620,13 +6615,13 @@
         <v>80</v>
       </c>
       <c r="E4" s="7" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="F4" s="7" t="s">
+        <v>190</v>
+      </c>
+      <c r="G4" s="7" t="s">
         <v>191</v>
-      </c>
-      <c r="G4" s="7" t="s">
-        <v>192</v>
       </c>
       <c r="H4" s="7">
         <v>11.001</v>
@@ -6655,7 +6650,7 @@
     </row>
     <row r="5" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A5" s="9" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="B5" s="7"/>
       <c r="C5" s="7" t="s">
@@ -6665,13 +6660,13 @@
         <v>80</v>
       </c>
       <c r="E5" s="7" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="F5" s="7" t="s">
+        <v>193</v>
+      </c>
+      <c r="G5" s="7" t="s">
         <v>194</v>
-      </c>
-      <c r="G5" s="7" t="s">
-        <v>195</v>
       </c>
       <c r="H5" s="7"/>
       <c r="I5" s="1">
@@ -6698,7 +6693,7 @@
     </row>
     <row r="6" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A6" s="9" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="B6" s="7" t="b">
         <v>1</v>
@@ -6710,13 +6705,13 @@
         <v>80</v>
       </c>
       <c r="E6" s="7" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="F6" s="7" t="s">
+        <v>196</v>
+      </c>
+      <c r="G6" s="7" t="s">
         <v>197</v>
-      </c>
-      <c r="G6" s="7" t="s">
-        <v>198</v>
       </c>
       <c r="H6" s="7">
         <v>3.001</v>
@@ -6726,18 +6721,18 @@
       </c>
       <c r="J6" s="25"/>
       <c r="K6" s="25" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="L6" s="25" t="s">
+        <v>198</v>
+      </c>
+      <c r="M6" s="25" t="s">
         <v>199</v>
-      </c>
-      <c r="M6" s="25" t="s">
-        <v>200</v>
       </c>
       <c r="N6" s="25"/>
       <c r="O6" s="25"/>
       <c r="P6" s="26" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="Q6" s="25"/>
       <c r="R6" s="25"/>
@@ -6753,7 +6748,7 @@
     </row>
     <row r="7" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A7" s="9" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="B7" s="7" t="b">
         <v>1</v>
@@ -6765,13 +6760,13 @@
         <v>80</v>
       </c>
       <c r="E7" s="7" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="F7" s="7" t="s">
+        <v>202</v>
+      </c>
+      <c r="G7" s="7" t="s">
         <v>203</v>
-      </c>
-      <c r="G7" s="7" t="s">
-        <v>204</v>
       </c>
       <c r="H7" s="7">
         <v>3.001</v>
@@ -6781,18 +6776,18 @@
       </c>
       <c r="J7" s="25"/>
       <c r="K7" s="25" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="L7" s="25" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="M7" s="25" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="N7" s="25"/>
       <c r="O7" s="25"/>
       <c r="P7" s="26" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="Q7" s="25"/>
       <c r="R7" s="25"/>
@@ -6808,7 +6803,7 @@
     </row>
     <row r="8" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A8" s="9" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="B8" s="7" t="b">
         <v>1</v>
@@ -6820,13 +6815,13 @@
         <v>80</v>
       </c>
       <c r="E8" s="7" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="F8" s="7" t="s">
+        <v>207</v>
+      </c>
+      <c r="G8" s="7" t="s">
         <v>208</v>
-      </c>
-      <c r="G8" s="7" t="s">
-        <v>209</v>
       </c>
       <c r="H8" s="7">
         <v>2.001</v>
@@ -6836,18 +6831,18 @@
       </c>
       <c r="J8" s="25"/>
       <c r="K8" s="25" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="L8" s="25" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="M8" s="25" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="N8" s="25"/>
       <c r="O8" s="25"/>
       <c r="P8" s="26" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="Q8" s="25"/>
       <c r="R8" s="25"/>
@@ -6863,7 +6858,7 @@
     </row>
     <row r="9" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A9" s="9" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="B9" s="7" t="b">
         <v>1</v>
@@ -6875,13 +6870,13 @@
         <v>80</v>
       </c>
       <c r="E9" s="7" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="F9" s="7" t="s">
+        <v>212</v>
+      </c>
+      <c r="G9" s="7" t="s">
         <v>213</v>
-      </c>
-      <c r="G9" s="7" t="s">
-        <v>214</v>
       </c>
       <c r="H9" s="7">
         <v>3.002</v>
@@ -6891,18 +6886,18 @@
       </c>
       <c r="J9" s="25"/>
       <c r="K9" s="25" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="L9" s="25" t="s">
+        <v>214</v>
+      </c>
+      <c r="M9" s="25" t="s">
         <v>215</v>
-      </c>
-      <c r="M9" s="25" t="s">
-        <v>216</v>
       </c>
       <c r="N9" s="25"/>
       <c r="O9" s="25"/>
       <c r="P9" s="26" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="Q9" s="25"/>
       <c r="R9" s="25"/>
@@ -6918,7 +6913,7 @@
     </row>
     <row r="10" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A10" s="9" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="B10" s="7" t="b">
         <v>1</v>
@@ -6930,13 +6925,13 @@
         <v>80</v>
       </c>
       <c r="E10" s="7" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="F10" s="7" t="s">
+        <v>218</v>
+      </c>
+      <c r="G10" s="7" t="s">
         <v>219</v>
-      </c>
-      <c r="G10" s="7" t="s">
-        <v>220</v>
       </c>
       <c r="H10" s="7">
         <v>3.002</v>
@@ -6946,18 +6941,18 @@
       </c>
       <c r="J10" s="25"/>
       <c r="K10" s="25" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="L10" s="25" t="s">
+        <v>220</v>
+      </c>
+      <c r="M10" s="25" t="s">
         <v>221</v>
-      </c>
-      <c r="M10" s="25" t="s">
-        <v>222</v>
       </c>
       <c r="N10" s="25"/>
       <c r="O10" s="25"/>
       <c r="P10" s="26" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="Q10" s="25"/>
       <c r="R10" s="25"/>
@@ -7361,7 +7356,7 @@
       <c r="J1" s="21"/>
       <c r="K1" s="22"/>
       <c r="L1" s="23" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="M1" s="24"/>
       <c r="N1" s="24"/>
@@ -7369,7 +7364,7 @@
       <c r="P1" s="24"/>
       <c r="Q1" s="24"/>
       <c r="R1" s="23" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="S1" s="24"/>
       <c r="T1" s="24"/>
@@ -7377,12 +7372,12 @@
       <c r="V1" s="24"/>
       <c r="W1" s="24"/>
       <c r="X1" s="23" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="Y1" s="24"/>
       <c r="Z1" s="24"/>
       <c r="AA1" s="23" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="AB1" s="24"/>
       <c r="AC1" s="24"/>
@@ -7402,7 +7397,7 @@
         <v>107</v>
       </c>
       <c r="B2" s="7" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="C2" s="7" t="s">
         <v>43</v>
@@ -7420,52 +7415,52 @@
         <v>110</v>
       </c>
       <c r="H2" s="7" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="I2" s="7" t="s">
+        <v>143</v>
+      </c>
+      <c r="J2" s="7" t="s">
         <v>144</v>
       </c>
-      <c r="J2" s="7" t="s">
+      <c r="K2" s="1" t="s">
         <v>145</v>
       </c>
-      <c r="K2" s="1" t="s">
-        <v>146</v>
-      </c>
       <c r="L2" s="19" t="s">
+        <v>225</v>
+      </c>
+      <c r="M2" s="7" t="s">
         <v>226</v>
       </c>
-      <c r="M2" s="7" t="s">
+      <c r="N2" s="7" t="s">
+        <v>147</v>
+      </c>
+      <c r="O2" s="7" t="s">
+        <v>120</v>
+      </c>
+      <c r="P2" s="7" t="s">
+        <v>121</v>
+      </c>
+      <c r="Q2" s="1" t="s">
+        <v>148</v>
+      </c>
+      <c r="R2" s="19" t="s">
         <v>227</v>
       </c>
-      <c r="N2" s="7" t="s">
-        <v>148</v>
-      </c>
-      <c r="O2" s="7" t="s">
-        <v>121</v>
-      </c>
-      <c r="P2" s="7" t="s">
-        <v>122</v>
-      </c>
-      <c r="Q2" s="1" t="s">
-        <v>149</v>
-      </c>
-      <c r="R2" s="19" t="s">
+      <c r="S2" s="7" t="s">
         <v>228</v>
       </c>
-      <c r="S2" s="7" t="s">
+      <c r="T2" s="7" t="s">
         <v>229</v>
       </c>
-      <c r="T2" s="7" t="s">
+      <c r="U2" s="7" t="s">
         <v>230</v>
       </c>
-      <c r="U2" s="7" t="s">
+      <c r="V2" s="7" t="s">
         <v>231</v>
       </c>
-      <c r="V2" s="7" t="s">
+      <c r="W2" s="1" t="s">
         <v>232</v>
-      </c>
-      <c r="W2" s="1" t="s">
-        <v>233</v>
       </c>
       <c r="X2" s="19" t="s">
         <v>54</v>
@@ -7495,24 +7490,24 @@
         <v>63</v>
       </c>
       <c r="AG2" s="19" t="s">
+        <v>233</v>
+      </c>
+      <c r="AH2" s="7" t="s">
         <v>234</v>
       </c>
-      <c r="AH2" s="7" t="s">
+      <c r="AI2" s="7" t="s">
         <v>235</v>
       </c>
-      <c r="AI2" s="7" t="s">
+      <c r="AJ2" s="7" t="s">
         <v>236</v>
       </c>
-      <c r="AJ2" s="7" t="s">
-        <v>237</v>
-      </c>
       <c r="AK2" s="1" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
     </row>
     <row r="3" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A3" s="9" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="B3" s="1" t="b">
         <v>0</v>
@@ -7524,43 +7519,43 @@
         <v>91</v>
       </c>
       <c r="E3" t="s">
+        <v>238</v>
+      </c>
+      <c r="F3" t="s">
         <v>239</v>
       </c>
-      <c r="F3" t="s">
+      <c r="G3" t="s">
         <v>240</v>
-      </c>
-      <c r="G3" t="s">
-        <v>241</v>
       </c>
       <c r="H3">
         <v>5.012</v>
       </c>
       <c r="I3" t="s">
+        <v>241</v>
+      </c>
+      <c r="J3" t="s">
+        <v>158</v>
+      </c>
+      <c r="K3" s="27" t="s">
         <v>242</v>
       </c>
-      <c r="J3" t="s">
-        <v>159</v>
-      </c>
-      <c r="K3" s="27" t="s">
+      <c r="L3" s="28" t="s">
         <v>243</v>
-      </c>
-      <c r="L3" s="28" t="s">
-        <v>244</v>
       </c>
       <c r="M3" s="14" t="s">
         <v>91</v>
       </c>
       <c r="N3" s="14" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="O3" s="14" t="s">
+        <v>168</v>
+      </c>
+      <c r="P3" s="14" t="s">
         <v>169</v>
       </c>
-      <c r="P3" s="14" t="s">
-        <v>170</v>
-      </c>
       <c r="Q3" s="29" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="R3" s="30" t="s">
         <v>91</v>
@@ -7571,10 +7566,10 @@
       <c r="AA3" s="30"/>
       <c r="AF3" s="27"/>
       <c r="AG3" s="30" t="s">
+        <v>245</v>
+      </c>
+      <c r="AH3" s="1" t="s">
         <v>246</v>
-      </c>
-      <c r="AH3" s="1" t="s">
-        <v>247</v>
       </c>
       <c r="AI3" s="1"/>
       <c r="AJ3" s="1"/>
@@ -7582,7 +7577,7 @@
     </row>
     <row r="4" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A4" s="9" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="B4" s="1" t="b">
         <v>0</v>
@@ -7594,43 +7589,43 @@
         <v>91</v>
       </c>
       <c r="E4" t="s">
+        <v>248</v>
+      </c>
+      <c r="F4" t="s">
         <v>249</v>
       </c>
-      <c r="F4" t="s">
-        <v>250</v>
-      </c>
       <c r="G4" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="H4">
         <v>5.012</v>
       </c>
       <c r="I4" t="s">
+        <v>250</v>
+      </c>
+      <c r="J4" t="s">
+        <v>158</v>
+      </c>
+      <c r="K4" s="27" t="s">
         <v>251</v>
       </c>
-      <c r="J4" t="s">
-        <v>159</v>
-      </c>
-      <c r="K4" s="27" t="s">
-        <v>252</v>
-      </c>
       <c r="L4" s="28" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="M4" s="14" t="s">
         <v>91</v>
       </c>
       <c r="N4" s="14" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="O4" s="14" t="s">
+        <v>168</v>
+      </c>
+      <c r="P4" s="14" t="s">
         <v>169</v>
       </c>
-      <c r="P4" s="14" t="s">
-        <v>170</v>
-      </c>
       <c r="Q4" s="29" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="R4" s="30" t="s">
         <v>91</v>
@@ -7641,10 +7636,10 @@
       <c r="AA4" s="30"/>
       <c r="AF4" s="27"/>
       <c r="AG4" s="30" t="s">
+        <v>253</v>
+      </c>
+      <c r="AH4" s="1" t="s">
         <v>254</v>
-      </c>
-      <c r="AH4" s="1" t="s">
-        <v>255</v>
       </c>
       <c r="AI4" s="1"/>
       <c r="AJ4" s="1"/>
@@ -7698,10 +7693,10 @@
   <sheetData>
     <row r="1" ht="15.75" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
+        <v>255</v>
+      </c>
+      <c r="M1" s="31" t="s">
         <v>256</v>
-      </c>
-      <c r="M1" s="31" t="s">
-        <v>257</v>
       </c>
       <c r="N1" s="32"/>
       <c r="O1" s="32"/>
@@ -7728,12 +7723,12 @@
       <c r="K2" s="35"/>
       <c r="L2" s="36"/>
       <c r="M2" s="37" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="N2" s="38"/>
       <c r="O2" s="39"/>
       <c r="P2" s="37" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="Q2" s="38"/>
       <c r="R2" s="38"/>
@@ -7756,7 +7751,7 @@
         <v>107</v>
       </c>
       <c r="B3" s="44" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="C3" s="44" t="s">
         <v>43</v>
@@ -7774,16 +7769,16 @@
         <v>110</v>
       </c>
       <c r="H3" s="45" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="I3" s="45" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="J3" s="45" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="K3" s="45" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="L3" s="45" t="s">
         <v>111</v>
@@ -7816,33 +7811,33 @@
         <v>63</v>
       </c>
       <c r="V3" s="43" t="s">
+        <v>261</v>
+      </c>
+      <c r="W3" s="44" t="s">
         <v>262</v>
       </c>
-      <c r="W3" s="44" t="s">
+      <c r="X3" s="44" t="s">
         <v>263</v>
       </c>
-      <c r="X3" s="44" t="s">
+      <c r="Y3" s="44" t="s">
         <v>264</v>
       </c>
-      <c r="Y3" s="44" t="s">
+      <c r="Z3" s="44" t="s">
         <v>265</v>
       </c>
-      <c r="Z3" s="44" t="s">
+      <c r="AA3" s="45" t="s">
         <v>266</v>
       </c>
-      <c r="AA3" s="45" t="s">
+      <c r="AB3" s="46" t="s">
         <v>267</v>
       </c>
-      <c r="AB3" s="46" t="s">
+      <c r="AC3" s="44" t="s">
         <v>268</v>
-      </c>
-      <c r="AC3" s="44" t="s">
-        <v>269</v>
       </c>
     </row>
     <row r="4" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A4" s="9" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="B4" s="48" t="b">
         <v>1</v>
@@ -7854,22 +7849,22 @@
         <v>91</v>
       </c>
       <c r="E4" s="48" t="s">
+        <v>270</v>
+      </c>
+      <c r="F4" s="49" t="s">
         <v>271</v>
       </c>
-      <c r="F4" s="49" t="s">
+      <c r="G4" s="49" t="s">
         <v>272</v>
-      </c>
-      <c r="G4" s="49" t="s">
-        <v>273</v>
       </c>
       <c r="H4" s="49">
         <v>5.001</v>
       </c>
       <c r="I4" s="49" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="J4" s="49" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="K4" s="49"/>
       <c r="L4" s="49"/>
@@ -7883,15 +7878,15 @@
       <c r="T4" s="49"/>
       <c r="U4" s="49"/>
       <c r="V4" s="50" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="W4" s="48"/>
       <c r="X4" s="48"/>
       <c r="Y4" s="48" t="s">
+        <v>275</v>
+      </c>
+      <c r="Z4" s="48" t="s">
         <v>276</v>
-      </c>
-      <c r="Z4" s="48" t="s">
-        <v>277</v>
       </c>
       <c r="AA4" s="49"/>
       <c r="AB4" s="49"/>
@@ -7899,7 +7894,7 @@
     </row>
     <row r="5" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A5" s="9" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="B5" s="48" t="b">
         <v>1</v>
@@ -7911,22 +7906,22 @@
         <v>91</v>
       </c>
       <c r="E5" s="48" t="s">
+        <v>278</v>
+      </c>
+      <c r="F5" s="49" t="s">
         <v>279</v>
       </c>
-      <c r="F5" s="49" t="s">
+      <c r="G5" s="49" t="s">
         <v>280</v>
-      </c>
-      <c r="G5" s="49" t="s">
-        <v>281</v>
       </c>
       <c r="H5" s="49">
         <v>5.001</v>
       </c>
       <c r="I5" s="49" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="J5" s="49" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="K5" s="49"/>
       <c r="L5" s="49"/>
@@ -7940,15 +7935,15 @@
       <c r="T5" s="49"/>
       <c r="U5" s="49"/>
       <c r="V5" s="50" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="W5" s="48"/>
       <c r="X5" s="48"/>
       <c r="Y5" s="48" t="s">
+        <v>282</v>
+      </c>
+      <c r="Z5" s="48" t="s">
         <v>283</v>
-      </c>
-      <c r="Z5" s="48" t="s">
-        <v>284</v>
       </c>
       <c r="AA5" s="49"/>
       <c r="AB5" s="49"/>
@@ -7956,7 +7951,7 @@
     </row>
     <row r="6" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A6" s="9" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="B6" s="48" t="b">
         <v>1</v>
@@ -7968,22 +7963,22 @@
         <v>102</v>
       </c>
       <c r="E6" s="48" t="s">
+        <v>285</v>
+      </c>
+      <c r="F6" s="49" t="s">
         <v>286</v>
       </c>
-      <c r="F6" s="49" t="s">
+      <c r="G6" s="49" t="s">
         <v>287</v>
       </c>
-      <c r="G6" s="49" t="s">
+      <c r="H6" s="49" t="s">
         <v>288</v>
       </c>
-      <c r="H6" s="49" t="s">
+      <c r="I6" s="49" t="s">
         <v>289</v>
       </c>
-      <c r="I6" s="49" t="s">
-        <v>290</v>
-      </c>
       <c r="J6" s="49" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="K6" s="49"/>
       <c r="L6" s="49"/>
@@ -8005,7 +8000,7 @@
         <v>85</v>
       </c>
       <c r="Z6" s="48" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="AA6" s="49"/>
       <c r="AB6" s="49"/>
@@ -8074,23 +8069,23 @@
       <c r="K1" s="16"/>
       <c r="L1" s="15"/>
       <c r="M1" s="16" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="N1" s="17"/>
       <c r="O1" s="17"/>
       <c r="P1" s="17"/>
       <c r="Q1" s="18"/>
       <c r="R1" s="16" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="S1" s="17"/>
       <c r="T1" s="16" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="U1" s="17"/>
       <c r="V1" s="18"/>
       <c r="W1" s="16" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="X1" s="17"/>
       <c r="Y1" s="17"/>
@@ -8107,10 +8102,10 @@
     </row>
     <row r="2" ht="45" customHeight="1" spans="1:33" s="7" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A2" s="19" t="s">
+        <v>293</v>
+      </c>
+      <c r="B2" s="7" t="s">
         <v>294</v>
-      </c>
-      <c r="B2" s="7" t="s">
-        <v>295</v>
       </c>
       <c r="C2" s="7" t="s">
         <v>43</v>
@@ -8119,43 +8114,43 @@
         <v>44</v>
       </c>
       <c r="E2" s="7" t="s">
+        <v>295</v>
+      </c>
+      <c r="F2" s="7" t="s">
         <v>296</v>
-      </c>
-      <c r="F2" s="7" t="s">
-        <v>297</v>
       </c>
       <c r="G2" s="7" t="s">
         <v>45</v>
       </c>
       <c r="H2" s="7" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="I2" s="7" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="J2" s="7" t="s">
+        <v>143</v>
+      </c>
+      <c r="K2" s="7" t="s">
         <v>144</v>
       </c>
-      <c r="K2" s="7" t="s">
+      <c r="L2" s="7" t="s">
         <v>145</v>
       </c>
-      <c r="L2" s="7" t="s">
+      <c r="M2" s="19" t="s">
         <v>146</v>
       </c>
-      <c r="M2" s="19" t="s">
+      <c r="N2" s="7" t="s">
         <v>147</v>
       </c>
-      <c r="N2" s="7" t="s">
+      <c r="O2" s="7" t="s">
+        <v>120</v>
+      </c>
+      <c r="P2" s="7" t="s">
+        <v>121</v>
+      </c>
+      <c r="Q2" s="1" t="s">
         <v>148</v>
-      </c>
-      <c r="O2" s="7" t="s">
-        <v>121</v>
-      </c>
-      <c r="P2" s="7" t="s">
-        <v>122</v>
-      </c>
-      <c r="Q2" s="1" t="s">
-        <v>149</v>
       </c>
       <c r="R2" s="19" t="s">
         <v>54</v>
@@ -8164,13 +8159,13 @@
         <v>55</v>
       </c>
       <c r="T2" s="19" t="s">
+        <v>298</v>
+      </c>
+      <c r="U2" s="7" t="s">
         <v>299</v>
       </c>
-      <c r="U2" s="7" t="s">
+      <c r="V2" s="1" t="s">
         <v>300</v>
-      </c>
-      <c r="V2" s="1" t="s">
-        <v>301</v>
       </c>
       <c r="W2" s="19" t="s">
         <v>58</v>
@@ -8191,24 +8186,24 @@
         <v>63</v>
       </c>
       <c r="AC2" s="19" t="s">
+        <v>301</v>
+      </c>
+      <c r="AD2" s="7" t="s">
+        <v>150</v>
+      </c>
+      <c r="AE2" s="7" t="s">
         <v>302</v>
       </c>
-      <c r="AD2" s="7" t="s">
-        <v>151</v>
-      </c>
-      <c r="AE2" s="7" t="s">
-        <v>303</v>
-      </c>
       <c r="AF2" s="7" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="AG2" s="1" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
     </row>
     <row r="3" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A3" s="9" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="B3" s="8" t="b">
         <v>1</v>
@@ -8220,35 +8215,35 @@
         <v>80</v>
       </c>
       <c r="E3" t="s">
+        <v>304</v>
+      </c>
+      <c r="F3" t="s">
         <v>305</v>
       </c>
-      <c r="F3" t="s">
+      <c r="G3" t="s">
         <v>306</v>
       </c>
-      <c r="G3" t="s">
+      <c r="H3" t="s">
         <v>307</v>
       </c>
-      <c r="H3" t="s">
+      <c r="I3" t="s">
         <v>308</v>
       </c>
-      <c r="I3" t="s">
+      <c r="J3" t="s">
         <v>309</v>
       </c>
-      <c r="J3" t="s">
-        <v>310</v>
-      </c>
       <c r="K3" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="M3" s="30" t="s">
+        <v>136</v>
+      </c>
+      <c r="N3" t="s">
         <v>137</v>
-      </c>
-      <c r="N3" t="s">
-        <v>138</v>
       </c>
       <c r="Q3" s="27"/>
       <c r="R3" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="S3" t="s">
         <v>88</v>
@@ -8265,7 +8260,7 @@
     </row>
     <row r="4" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A4" s="9" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="B4" s="8" t="b">
         <v>0</v>
@@ -8277,46 +8272,46 @@
         <v>91</v>
       </c>
       <c r="E4" t="s">
+        <v>312</v>
+      </c>
+      <c r="F4" t="s">
         <v>313</v>
       </c>
-      <c r="F4" t="s">
+      <c r="G4" t="s">
         <v>314</v>
       </c>
-      <c r="G4" t="s">
+      <c r="H4" t="s">
         <v>315</v>
-      </c>
-      <c r="H4" t="s">
-        <v>316</v>
       </c>
       <c r="I4">
         <v>11.001</v>
       </c>
       <c r="J4" t="s">
+        <v>316</v>
+      </c>
+      <c r="K4" t="s">
+        <v>158</v>
+      </c>
+      <c r="L4" t="s">
         <v>317</v>
       </c>
-      <c r="K4" t="s">
-        <v>159</v>
-      </c>
-      <c r="L4" t="s">
+      <c r="M4" s="30" t="s">
+        <v>136</v>
+      </c>
+      <c r="N4" t="s">
+        <v>137</v>
+      </c>
+      <c r="O4" t="s">
+        <v>168</v>
+      </c>
+      <c r="P4" t="s">
+        <v>169</v>
+      </c>
+      <c r="Q4" s="27" t="s">
         <v>318</v>
       </c>
-      <c r="M4" s="30" t="s">
-        <v>137</v>
-      </c>
-      <c r="N4" t="s">
-        <v>138</v>
-      </c>
-      <c r="O4" t="s">
-        <v>169</v>
-      </c>
-      <c r="P4" t="s">
-        <v>170</v>
-      </c>
-      <c r="Q4" s="27" t="s">
+      <c r="R4" t="s">
         <v>319</v>
-      </c>
-      <c r="R4" t="s">
-        <v>320</v>
       </c>
       <c r="S4" t="s">
         <v>88</v>
@@ -8403,39 +8398,39 @@
         <v>108</v>
       </c>
       <c r="E2" s="7" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
       <c r="F2" s="7" t="s">
         <v>45</v>
       </c>
       <c r="G2" s="7" t="s">
+        <v>378</v>
+      </c>
+      <c r="H2" s="7" t="s">
         <v>379</v>
       </c>
-      <c r="H2" s="7" t="s">
+      <c r="I2" s="7" t="s">
         <v>380</v>
       </c>
-      <c r="I2" s="7" t="s">
+      <c r="J2" s="7" t="s">
         <v>381</v>
       </c>
-      <c r="J2" s="7" t="s">
-        <v>382</v>
-      </c>
       <c r="K2" s="4" t="s">
+        <v>122</v>
+      </c>
+      <c r="L2" s="7" t="s">
         <v>123</v>
-      </c>
-      <c r="L2" s="7" t="s">
-        <v>124</v>
       </c>
       <c r="M2" s="7" t="s">
         <v>110</v>
       </c>
       <c r="N2" s="8" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
     </row>
     <row r="3" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A3" s="9" t="s">
-        <v>383</v>
+        <v>382</v>
       </c>
       <c r="B3" t="s">
         <v>90</v>
@@ -8444,19 +8439,19 @@
         <v>91</v>
       </c>
       <c r="D3" t="s">
+        <v>383</v>
+      </c>
+      <c r="E3" t="s">
         <v>384</v>
       </c>
-      <c r="E3" t="s">
+      <c r="F3" t="s">
         <v>385</v>
       </c>
-      <c r="F3" t="s">
+      <c r="G3" t="s">
         <v>386</v>
       </c>
-      <c r="G3" t="s">
+      <c r="H3" t="s">
         <v>387</v>
-      </c>
-      <c r="H3" t="s">
-        <v>388</v>
       </c>
       <c r="I3">
         <v>3</v>
@@ -8471,7 +8466,7 @@
     </row>
     <row r="4" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A4" s="9" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="B4" t="s">
         <v>90</v>
@@ -8480,19 +8475,19 @@
         <v>91</v>
       </c>
       <c r="D4" t="s">
-        <v>384</v>
+        <v>383</v>
       </c>
       <c r="E4" t="s">
+        <v>389</v>
+      </c>
+      <c r="F4" t="s">
         <v>390</v>
       </c>
-      <c r="F4" t="s">
+      <c r="G4" t="s">
         <v>391</v>
       </c>
-      <c r="G4" t="s">
+      <c r="H4" t="s">
         <v>392</v>
-      </c>
-      <c r="H4" t="s">
-        <v>393</v>
       </c>
       <c r="I4">
         <v>4</v>

</xml_diff>